<commit_message>
loss and revenue are now coloered red/green. added ETFs/Stocks to account name. added 9.10.24 deposit.
</commit_message>
<xml_diff>
--- a/ExcelFiles/Deposits.xlsx
+++ b/ExcelFiles/Deposits.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danagershon/Documents/Investing/ExcelFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A7938E1-C78C-C545-824E-D5078CD1700B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2FD2040-3649-7C49-ABE6-6D7B3EC16528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="25440" xr2:uid="{01897C2D-4096-C442-BFA4-715938F33431}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="6">
   <si>
     <t>Amount</t>
   </si>
@@ -935,7 +935,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D61DA251-10CA-4844-BBF4-8AEDC623E4A8}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.85546875" style="5" customWidth="1"/>
@@ -1056,6 +1056,20 @@
         <v>3</v>
       </c>
     </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="5">
+        <v>45574</v>
+      </c>
+      <c r="B9" s="6">
+        <v>23000</v>
+      </c>
+      <c r="C9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D9" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>